<commit_message>
Fixed bound on industry fuels shares and add dummy import limits
</commit_message>
<xml_diff>
--- a/SysSettings.xlsx
+++ b/SysSettings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BB1EBD-AD17-47CD-994B-6C52298E6487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D7E432-BBD3-4827-B824-DED810952E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="28" r:id="rId1"/>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="170">
   <si>
     <t>~TFM_UPD</t>
   </si>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C3" s="11"/>
     </row>
-    <row r="4" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2018</v>
       </c>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C7" s="11"/>
     </row>
-    <row r="8" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>37</v>
       </c>
@@ -7899,7 +7899,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="13" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" s="12">
         <v>1</v>
       </c>
@@ -7971,7 +7971,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="14" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" s="12">
         <v>1</v>
       </c>
@@ -8043,7 +8043,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="15" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" s="12">
         <v>1</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="16" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" s="12">
         <v>20</v>
       </c>
@@ -8187,7 +8187,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="17" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B17" s="12">
         <v>20</v>
       </c>
@@ -8259,7 +8259,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="18" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C18" s="12">
         <v>5</v>
       </c>
@@ -8324,7 +8324,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="19" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C19" s="12">
         <v>45</v>
       </c>
@@ -8389,7 +8389,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="20" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C20" s="12">
         <v>25</v>
       </c>
@@ -8454,7 +8454,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="21" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C21" s="12">
         <v>5</v>
       </c>
@@ -8519,7 +8519,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="22" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="D22" s="12">
         <v>5</v>
       </c>
@@ -8577,7 +8577,7 @@
         <v>2029</v>
       </c>
     </row>
-    <row r="23" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="D23" s="12">
         <v>5</v>
       </c>
@@ -8635,7 +8635,7 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="24" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="D24" s="12">
         <v>5</v>
       </c>
@@ -8693,7 +8693,7 @@
         <v>2039</v>
       </c>
     </row>
-    <row r="25" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E25" s="12">
         <v>5</v>
       </c>
@@ -8744,7 +8744,7 @@
         <v>2044</v>
       </c>
     </row>
-    <row r="26" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="F26" s="12">
         <v>5</v>
       </c>
@@ -8788,7 +8788,7 @@
         <v>2049</v>
       </c>
     </row>
-    <row r="27" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="F27" s="12">
         <v>5</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>2054</v>
       </c>
     </row>
-    <row r="28" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="G28" s="12">
         <v>5</v>
       </c>
@@ -8869,7 +8869,7 @@
         <v>2059</v>
       </c>
     </row>
-    <row r="29" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="G29" s="12">
         <v>5</v>
       </c>
@@ -8899,7 +8899,7 @@
         <v>2064</v>
       </c>
     </row>
-    <row r="30" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="G30" s="12">
         <v>5</v>
       </c>
@@ -8929,7 +8929,7 @@
         <v>2069</v>
       </c>
     </row>
-    <row r="31" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="G31" s="12">
         <v>5</v>
       </c>
@@ -8959,7 +8959,7 @@
         <v>2074</v>
       </c>
     </row>
-    <row r="32" spans="2:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="G32" s="12">
         <v>5</v>
       </c>
@@ -8989,7 +8989,7 @@
         <v>2079</v>
       </c>
     </row>
-    <row r="33" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:22" x14ac:dyDescent="0.25">
       <c r="G33" s="12">
         <v>5</v>
       </c>
@@ -9019,7 +9019,7 @@
         <v>2084</v>
       </c>
     </row>
-    <row r="34" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:22" x14ac:dyDescent="0.25">
       <c r="G34" s="12">
         <v>5</v>
       </c>
@@ -9049,7 +9049,7 @@
         <v>2089</v>
       </c>
     </row>
-    <row r="35" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:22" x14ac:dyDescent="0.25">
       <c r="G35" s="12">
         <v>5</v>
       </c>
@@ -9079,7 +9079,7 @@
         <v>2094</v>
       </c>
     </row>
-    <row r="36" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H36" s="17">
         <v>1</v>
       </c>
@@ -9102,7 +9102,7 @@
         <v>2099</v>
       </c>
     </row>
-    <row r="37" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H37" s="17">
         <v>1</v>
       </c>
@@ -9118,7 +9118,7 @@
         <v>2042</v>
       </c>
     </row>
-    <row r="38" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H38" s="17">
         <v>1</v>
       </c>
@@ -9134,7 +9134,7 @@
         <v>2043</v>
       </c>
     </row>
-    <row r="39" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H39" s="17">
         <v>1</v>
       </c>
@@ -9150,7 +9150,7 @@
         <v>2044</v>
       </c>
     </row>
-    <row r="40" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H40" s="17">
         <v>1</v>
       </c>
@@ -9166,7 +9166,7 @@
         <v>2045</v>
       </c>
     </row>
-    <row r="41" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H41" s="17">
         <v>1</v>
       </c>
@@ -9182,7 +9182,7 @@
         <v>2046</v>
       </c>
     </row>
-    <row r="42" spans="7:22" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:22" x14ac:dyDescent="0.25">
       <c r="H42" s="17">
         <v>1</v>
       </c>
@@ -9330,7 +9330,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="17" t="s">
         <v>27</v>
       </c>
@@ -9338,7 +9338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>28</v>
       </c>
@@ -9346,7 +9346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>29</v>
       </c>
@@ -9354,7 +9354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>30</v>
       </c>
@@ -9362,7 +9362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="13.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>49</v>
       </c>
@@ -9784,7 +9784,7 @@
       <c r="H22" s="24"/>
       <c r="I22" s="24"/>
       <c r="J22" s="24" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K22" s="24"/>
       <c r="L22" s="24"/>
@@ -9796,14 +9796,22 @@
     <row r="23" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A23" s="24"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
+      <c r="C23" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" s="24">
+        <v>0</v>
+      </c>
       <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="F23" s="24">
+        <v>5</v>
+      </c>
       <c r="G23" s="24"/>
       <c r="H23" s="24"/>
       <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
+      <c r="J23" s="24" t="s">
+        <v>1</v>
+      </c>
       <c r="K23" s="24"/>
       <c r="L23" s="24"/>
       <c r="M23" s="24"/>

</xml_diff>